<commit_message>
docs: lead with audited scraper speed accuracy and token results
Feature the measured comparison before the demo in README, including a real chart, all ten paired results, per-run token breakdowns and reproducible evidence. Agent mean 40.0486s versus native workflow 6.1233s (6.54x); both 10/10 successful and 200/200 canonical fields correct. Agent mean 153304.4 reported model tokens per run including cached input, native repeat runs zero; exclude builder setup and avoid dollar-cost claims. Update the workbook with actual measurements, tested formulas and editable charts. Scope the claims to the headless local scraper and shared parser. Version 0.16.2 synchronized. 81 frontend tests, independent 20-run audit, workbook formula checks and Windows installer build passed.
</commit_message>
<xml_diff>
--- a/outputs/2026-10-30-mcp-comparison/mcp-workflow-comparison.xlsx
+++ b/outputs/2026-10-30-mcp-comparison/mcp-workflow-comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="1" r:id="R3b31e7c382bf43da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark" sheetId="2" r:id="Rbb7d01b3202042db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="1" r:id="R18bf33b258e04e43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark" sheetId="2" r:id="Rf8bbaeab469a4912"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,11 +14,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="0.0"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
     <x:numFmt numFmtId="202" formatCode="0.00&quot;x&quot;"/>
     <x:numFmt numFmtId="203" formatCode="0"/>
+    <x:numFmt numFmtId="204" formatCode="0.00"/>
+    <x:numFmt numFmtId="205" formatCode="#,##0"/>
+    <x:numFmt numFmtId="206" formatCode="#,##0.0"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -61,7 +64,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -83,6 +86,26 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F3EA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F3EA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245942"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F3EA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -96,7 +119,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -148,6 +171,58 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -364,6 +439,627 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr>
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:rPr>
+              <a:t>Mean scraper time (seconds), 10 runs each</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr>
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Prompt agent</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="83968B"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Comparison'!$G$3</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Comparison'!$H$3</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Saved workflow</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="245942"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Comparison'!$G$3</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Comparison'!$I$3</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900">
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr>
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:rPr>
+              <a:t>Observed field accuracy, 200 fields each</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr>
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Prompt agent</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="83968B"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Comparison'!$G$6</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Comparison'!$H$6</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Saved workflow</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="245942"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Comparison'!$G$6</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Comparison'!$I$6</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0%" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900">
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr>
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:rPr>
+              <a:t>Mean model tokens per run (includes cached input)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr>
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Prompt agent</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="83968B"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Comparison'!$G$40</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Comparison'!$H$40</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Saved workflow</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="245942"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Comparison'!$G$40</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Comparison'!$I$40</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900">
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -390,7 +1086,97 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R57efa2ec14e74888"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re271cd55082b4d50"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R469e483566d344be"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R04c43edd2c924cde"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R73cf55e225194e7d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -602,6 +1388,9 @@
     <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="31" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="21" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="21" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="21" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -617,40 +1406,57 @@
       <x:c r="J1" s="2"/>
       <x:c r="K1" s="2"/>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="2"/>
       <x:c r="B2" s="3" t="str">
-        <x:v>MCP agents and MCP Workflow</x:v>
+        <x:v>Measured results</x:v>
       </x:c>
       <x:c r="C2" s="2"/>
       <x:c r="D2" s="2"/>
       <x:c r="E2" s="2"/>
       <x:c r="F2" s="2"/>
-      <x:c r="G2" s="2"/>
-      <x:c r="H2" s="2"/>
-      <x:c r="I2" s="2"/>
+      <x:c r="G2" s="2" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="str">
+        <x:v>Prompt agent</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="str">
+        <x:v>Saved workflow</x:v>
+      </x:c>
       <x:c r="J2" s="2"/>
       <x:c r="K2" s="2"/>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="2"/>
       <x:c r="B3" s="4" t="str">
-        <x:v>As of October 30, 2026. App v0.16.0. Qualitative comparison, not a matched performance benchmark.</x:v>
-      </x:c>
-      <x:c r="C3" s="2"/>
+        <x:f>TEXT(Benchmark!G5,"0.00")&amp;"x faster"</x:f>
+        <x:v>6.54x faster</x:v>
+      </x:c>
+      <x:c r="C3" s="4" t="str">
+        <x:v>Both methods: 100% observed field accuracy.</x:v>
+      </x:c>
       <x:c r="D3" s="2"/>
       <x:c r="E3" s="2"/>
       <x:c r="F3" s="2"/>
-      <x:c r="G3" s="2"/>
-      <x:c r="H3" s="2"/>
-      <x:c r="I3" s="2"/>
+      <x:c r="G3" s="2" t="str">
+        <x:v>Mean elapsed (s)</x:v>
+      </x:c>
+      <x:c r="H3" s="21" t="n">
+        <x:f>Benchmark!C6</x:f>
+        <x:v>40.048610579999995</x:v>
+      </x:c>
+      <x:c r="I3" s="21" t="n">
+        <x:f>Benchmark!D6</x:f>
+        <x:v>6.123301240000009</x:v>
+      </x:c>
       <x:c r="J3" s="2"/>
       <x:c r="K3" s="2"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2"/>
       <x:c r="B4" s="4" t="str">
-        <x:v>Baseline: an agent given a saved prompt and MCP tools, without a separate saved executable workflow. Agent host features vary.</x:v>
+        <x:v>October 30, 2026. Ten paired local scraper cases. GPT-6.1 Sol, low reasoning. Native workflow needs no per-run model inference.</x:v>
       </x:c>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="2"/>
@@ -669,9 +1475,15 @@
       <x:c r="D5" s="2"/>
       <x:c r="E5" s="2"/>
       <x:c r="F5" s="2"/>
-      <x:c r="G5" s="2"/>
-      <x:c r="H5" s="2"/>
-      <x:c r="I5" s="2"/>
+      <x:c r="G5" s="2" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+      <x:c r="H5" s="2" t="str">
+        <x:v>Prompt agent</x:v>
+      </x:c>
+      <x:c r="I5" s="2" t="str">
+        <x:v>Saved workflow</x:v>
+      </x:c>
       <x:c r="J5" s="2"/>
       <x:c r="K5" s="2"/>
     </x:row>
@@ -690,9 +1502,17 @@
         <x:v>Interpretation</x:v>
       </x:c>
       <x:c r="F6" s="2"/>
-      <x:c r="G6" s="2"/>
-      <x:c r="H6" s="2"/>
-      <x:c r="I6" s="2"/>
+      <x:c r="G6" s="2" t="str">
+        <x:v>Field accuracy</x:v>
+      </x:c>
+      <x:c r="H6" s="14" t="n">
+        <x:f>Benchmark!C7</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I6" s="14" t="n">
+        <x:f>Benchmark!D7</x:f>
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="J6" s="2"/>
       <x:c r="K6" s="2"/>
     </x:row>
@@ -723,13 +1543,13 @@
         <x:v>Repeated run speed</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>May plan again on each run. A host can cache or reuse plans.</x:v>
+        <x:v>40.05 s mean with fresh prompt and MCP.</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Saved graph reuses the plan. Native steps skip model inference.</x:v>
+        <x:v>6.12 s mean with the saved native graph.</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>Expected benefit; not measured.</x:v>
+        <x:v>6.54x faster in this test.</x:v>
       </x:c>
       <x:c r="F8" s="2"/>
       <x:c r="G8" s="2"/>
@@ -765,13 +1585,13 @@
         <x:v>Output accuracy</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>Depends on model, instructions, tools and validation.</x:v>
+        <x:v>100%: 200/200 canonical fields, checked in both CSV and JSON.</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Native rules repeat configured logic; AI outputs still vary.</x:v>
+        <x:v>100%: 200/200 canonical fields, checked in both CSV and JSON.</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>No comparative accuracy rate yet.</x:v>
+        <x:v>No observed accuracy advantage.</x:v>
       </x:c>
       <x:c r="F10" s="2"/>
       <x:c r="G10" s="2"/>
@@ -786,13 +1606,13 @@
         <x:v>Accuracy when reused</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
-        <x:v>A saved prompt repeats intent; the agent may choose a different route.</x:v>
+        <x:v>5/5 changed-input cases correct with the same prompt.</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>Saved steps keep routing and fields. Bad rules repeat errors too.</x:v>
+        <x:v>5/5 changed-input cases correct with the same saved graph.</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>Better control does not prove correctness.</x:v>
+        <x:v>Input values changed; arbitrary page layouts were not tested.</x:v>
       </x:c>
       <x:c r="F11" s="2"/>
       <x:c r="G11" s="2"/>
@@ -975,13 +1795,13 @@
         <x:v>Cost and AI usage</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>Depends on inference calls, tools and subscription/API billing.</x:v>
+        <x:v>153,304.4 reported model tokens/run on average, including cached input.</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>Native steps use no model inference; builder and AI steps do.</x:v>
+        <x:v>0 model tokens per native repeat run. Builder/setup usage excluded.</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>No measured cost saving yet.</x:v>
+        <x:v>No dollar cost comparison. AI steps still consume model tokens.</x:v>
       </x:c>
       <x:c r="F20" s="2"/>
       <x:c r="G20" s="2"/>
@@ -1112,7 +1932,7 @@
     <x:row r="28">
       <x:c r="A28" s="2"/>
       <x:c r="B28" s="2" t="str">
-        <x:v>No prompt-agent baseline or controlled timing sample was collected. Video duration is not workflow execution time.</x:v>
+        <x:v>Matched result: ten trials per method, including six seconds of deliberate waits. One pilot was excluded on both sides.</x:v>
       </x:c>
       <x:c r="C28" s="2"/>
       <x:c r="D28" s="2"/>
@@ -1279,9 +2099,15 @@
       <x:c r="D39" s="2"/>
       <x:c r="E39" s="2"/>
       <x:c r="F39" s="2"/>
-      <x:c r="G39" s="2"/>
-      <x:c r="H39" s="2"/>
-      <x:c r="I39" s="2"/>
+      <x:c r="G39" s="2" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+      <x:c r="H39" s="2" t="str">
+        <x:v>Prompt agent</x:v>
+      </x:c>
+      <x:c r="I39" s="2" t="str">
+        <x:v>Saved workflow</x:v>
+      </x:c>
       <x:c r="J39" s="2"/>
       <x:c r="K39" s="2"/>
     </x:row>
@@ -1292,9 +2118,17 @@
       <x:c r="D40" s="2"/>
       <x:c r="E40" s="2"/>
       <x:c r="F40" s="2"/>
-      <x:c r="G40" s="2"/>
-      <x:c r="H40" s="2"/>
-      <x:c r="I40" s="2"/>
+      <x:c r="G40" s="2" t="str">
+        <x:v>Mean model tokens/run</x:v>
+      </x:c>
+      <x:c r="H40" s="38" t="n">
+        <x:f>Benchmark!C47</x:f>
+        <x:v>153304.4</x:v>
+      </x:c>
+      <x:c r="I40" s="38" t="n">
+        <x:f>Benchmark!D47</x:f>
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="J40" s="2"/>
       <x:c r="K40" s="2"/>
     </x:row>
@@ -1477,13 +2311,13 @@
     <x:row r="53" ht="46" customHeight="1">
       <x:c r="A53" s="2"/>
       <x:c r="B53" s="9" t="str">
-        <x:v>Interpretation</x:v>
+        <x:v>Measured evidence</x:v>
       </x:c>
       <x:c r="C53" s="9" t="str">
-        <x:v>Speed expectations above are engineering judgments, not benchmark results.</x:v>
+        <x:v>Independent audit, run ledger, files and fixture hashes</x:v>
       </x:c>
       <x:c r="D53" s="9" t="str">
-        <x:v>Use the Benchmark sheet for matched measurements.</x:v>
+        <x:v>benchmarks/results/measured-2026-10-30T08-02-42-177Z</x:v>
       </x:c>
       <x:c r="E53" s="9"/>
       <x:c r="F53" s="2"/>
@@ -1493,12 +2327,18 @@
       <x:c r="J53" s="2"/>
       <x:c r="K53" s="2"/>
     </x:row>
-    <x:row r="54">
+    <x:row r="54" ht="46" customHeight="1">
       <x:c r="A54" s="2"/>
-      <x:c r="B54" s="2"/>
-      <x:c r="C54" s="2"/>
-      <x:c r="D54" s="2"/>
-      <x:c r="E54" s="2"/>
+      <x:c r="B54" s="9" t="str">
+        <x:v>Limits</x:v>
+      </x:c>
+      <x:c r="C54" s="9" t="str">
+        <x:v>Headless native scraping only; excludes UI, setup authoring and AI-heavy workflows.</x:v>
+      </x:c>
+      <x:c r="D54" s="9" t="str">
+        <x:v>An agent reusing code or a higher-level tool is a different baseline.</x:v>
+      </x:c>
+      <x:c r="E54" s="9"/>
       <x:c r="F54" s="2"/>
       <x:c r="G54" s="2"/>
       <x:c r="H54" s="2"/>
@@ -1586,7 +2426,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6bcdfb3d8e54418"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4439c56654474dab"/>
 </x:worksheet>
 </file>
 
@@ -1606,6 +2446,10 @@
     <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="19" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="21" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="21" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="21" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1624,7 +2468,7 @@
     <x:row r="2">
       <x:c r="A2" s="2"/>
       <x:c r="B2" s="3" t="str">
-        <x:v>Matched benchmark worksheet</x:v>
+        <x:v>Measured scraper benchmark</x:v>
       </x:c>
       <x:c r="C2" s="2"/>
       <x:c r="D2" s="2"/>
@@ -1639,7 +2483,7 @@
     <x:row r="3">
       <x:c r="A3" s="2"/>
       <x:c r="B3" s="2" t="str">
-        <x:v>No results entered. Yellow cells are measurement inputs. Blank is unknown, not zero.</x:v>
+        <x:v>20 completed runs on October 30, 2026. Raw measurements below; formulas calculate the comparison above.</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -1679,8 +2523,9 @@
       <x:c r="F5" s="2" t="str">
         <x:v>Measured speedup</x:v>
       </x:c>
-      <x:c r="G5" s="15" t="str">
+      <x:c r="G5" s="15" t="n">
         <x:f>IF(OR(C6="",D6="",D6=0),"",C6/D6)</x:f>
+        <x:v>6.540362626353483</x:v>
       </x:c>
       <x:c r="H5" s="2"/>
       <x:c r="I5" s="2"/>
@@ -1692,11 +2537,13 @@
       <x:c r="B6" s="2" t="str">
         <x:v>Average elapsed time (s)</x:v>
       </x:c>
-      <x:c r="C6" s="13" t="str">
+      <x:c r="C6" s="21" t="n">
         <x:f>IF(COUNTIFS($B$15:$B$34,C$5,$D$15:$D$34,"&lt;&gt;",$D$15:$D$34,"&gt;=0")=0,"",SUMIFS($D$15:$D$34,$B$15:$B$34,C$5)/COUNTIFS($B$15:$B$34,C$5,$D$15:$D$34,"&lt;&gt;",$D$15:$D$34,"&gt;=0"))</x:f>
-      </x:c>
-      <x:c r="D6" s="13" t="str">
+        <x:v>40.048610579999995</x:v>
+      </x:c>
+      <x:c r="D6" s="21" t="n">
         <x:f>IF(COUNTIFS($B$15:$B$34,D$5,$D$15:$D$34,"&lt;&gt;",$D$15:$D$34,"&gt;=0")=0,"",SUMIFS($D$15:$D$34,$B$15:$B$34,D$5)/COUNTIFS($B$15:$B$34,D$5,$D$15:$D$34,"&lt;&gt;",$D$15:$D$34,"&gt;=0"))</x:f>
+        <x:v>6.123301240000009</x:v>
       </x:c>
       <x:c r="E6" s="2"/>
       <x:c r="F6" s="2"/>
@@ -1711,18 +2558,21 @@
       <x:c r="B7" s="2" t="str">
         <x:v>Field accuracy</x:v>
       </x:c>
-      <x:c r="C7" s="14" t="str">
+      <x:c r="C7" s="14" t="n">
         <x:f>IF(SUMIFS($F$15:$F$34,$B$15:$B$34,C$5)=0,"",SUMIFS($E$15:$E$34,$B$15:$B$34,C$5)/SUMIFS($F$15:$F$34,$B$15:$B$34,C$5))</x:f>
-      </x:c>
-      <x:c r="D7" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="n">
         <x:f>IF(SUMIFS($F$15:$F$34,$B$15:$B$34,D$5)=0,"",SUMIFS($E$15:$E$34,$B$15:$B$34,D$5)/SUMIFS($F$15:$F$34,$B$15:$B$34,D$5))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E7" s="2"/>
       <x:c r="F7" s="2" t="str">
         <x:v>Accuracy delta (pp)</x:v>
       </x:c>
-      <x:c r="G7" s="13" t="str">
+      <x:c r="G7" s="13" t="n">
         <x:f>IF(OR(C7="",D7=""),"",(D7-C7)*100)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="2"/>
       <x:c r="I7" s="2"/>
@@ -1734,11 +2584,13 @@
       <x:c r="B8" s="2" t="str">
         <x:v>Successful run rate</x:v>
       </x:c>
-      <x:c r="C8" s="14" t="str">
+      <x:c r="C8" s="14" t="n">
         <x:f>IF(COUNTIFS($B$15:$B$34,C$5,$G$15:$G$34,"&lt;&gt;",$G$15:$G$34,"&gt;=0")=0,"",SUMIFS($G$15:$G$34,$B$15:$B$34,C$5)/COUNTIFS($B$15:$B$34,C$5,$G$15:$G$34,"&lt;&gt;",$G$15:$G$34,"&gt;=0"))</x:f>
-      </x:c>
-      <x:c r="D8" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D8" s="14" t="n">
         <x:f>IF(COUNTIFS($B$15:$B$34,D$5,$G$15:$G$34,"&lt;&gt;",$G$15:$G$34,"&gt;=0")=0,"",SUMIFS($G$15:$G$34,$B$15:$B$34,D$5)/COUNTIFS($B$15:$B$34,D$5,$G$15:$G$34,"&lt;&gt;",$G$15:$G$34,"&gt;=0"))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E8" s="2"/>
       <x:c r="F8" s="2"/>
@@ -1753,11 +2605,13 @@
       <x:c r="B9" s="2" t="str">
         <x:v>Average human fixes</x:v>
       </x:c>
-      <x:c r="C9" s="13" t="str">
+      <x:c r="C9" s="13" t="n">
         <x:f>IF(COUNTIFS($B$15:$B$34,C$5,$H$15:$H$34,"&lt;&gt;",$H$15:$H$34,"&gt;=0")=0,"",SUMIFS($H$15:$H$34,$B$15:$B$34,C$5)/COUNTIFS($B$15:$B$34,C$5,$H$15:$H$34,"&lt;&gt;",$H$15:$H$34,"&gt;=0"))</x:f>
-      </x:c>
-      <x:c r="D9" s="13" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="13" t="n">
         <x:f>IF(COUNTIFS($B$15:$B$34,D$5,$H$15:$H$34,"&lt;&gt;",$H$15:$H$34,"&gt;=0")=0,"",SUMIFS($H$15:$H$34,$B$15:$B$34,D$5)/COUNTIFS($B$15:$B$34,D$5,$H$15:$H$34,"&lt;&gt;",$H$15:$H$34,"&gt;=0"))</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="2"/>
       <x:c r="F9" s="2"/>
@@ -1769,9 +2623,17 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2"/>
-      <x:c r="B10" s="2"/>
-      <x:c r="C10" s="2"/>
-      <x:c r="D10" s="2"/>
+      <x:c r="B10" s="2" t="str">
+        <x:v>Median elapsed time (s)</x:v>
+      </x:c>
+      <x:c r="C10" s="21" t="n">
+        <x:f>MEDIAN(D15,D17,D19,D21,D23,D25,D27,D29,D31,D33)</x:f>
+        <x:v>39.513275300000004</x:v>
+      </x:c>
+      <x:c r="D10" s="21" t="n">
+        <x:f>MEDIAN(D16,D18,D20,D22,D24,D26,D28,D30,D32,D34)</x:f>
+        <x:v>6.122887000000002</x:v>
+      </x:c>
       <x:c r="E10" s="2"/>
       <x:c r="F10" s="2"/>
       <x:c r="G10" s="2"/>
@@ -1783,10 +2645,16 @@
     <x:row r="11">
       <x:c r="A11" s="2"/>
       <x:c r="B11" s="2" t="str">
-        <x:v>Use the same model/version, tools, frozen inputs, expected fields, timeout and task. Alternate methods across 10 paired runs.</x:v>
-      </x:c>
-      <x:c r="C11" s="2"/>
-      <x:c r="D11" s="2"/>
+        <x:v>Minimum elapsed time (s)</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="n">
+        <x:f>MIN(D15,D17,D19,D21,D23,D25,D27,D29,D31,D33)</x:f>
+        <x:v>29.247441099999996</x:v>
+      </x:c>
+      <x:c r="D11" s="21" t="n">
+        <x:f>MIN(D16,D18,D20,D22,D24,D26,D28,D30,D32,D34)</x:f>
+        <x:v>6.096144200000002</x:v>
+      </x:c>
       <x:c r="E11" s="2"/>
       <x:c r="F11" s="2"/>
       <x:c r="G11" s="2"/>
@@ -1798,10 +2666,16 @@
     <x:row r="12">
       <x:c r="A12" s="2"/>
       <x:c r="B12" s="2" t="str">
-        <x:v>Measure setup separately. Time start-to-validated-file, including waits/retries. Keep failed runs and mark success 0.</x:v>
-      </x:c>
-      <x:c r="C12" s="2"/>
-      <x:c r="D12" s="2"/>
+        <x:v>Maximum elapsed time (s)</x:v>
+      </x:c>
+      <x:c r="C12" s="21" t="n">
+        <x:f>MAX(D15,D17,D19,D21,D23,D25,D27,D29,D31,D33)</x:f>
+        <x:v>55.79296789999999</x:v>
+      </x:c>
+      <x:c r="D12" s="21" t="n">
+        <x:f>MAX(D16,D18,D20,D22,D24,D26,D28,D30,D32,D34)</x:f>
+        <x:v>6.167543500000029</x:v>
+      </x:c>
       <x:c r="E12" s="2"/>
       <x:c r="F12" s="2"/>
       <x:c r="G12" s="2"/>
@@ -1847,10 +2721,20 @@
         <x:v>Human fixes</x:v>
       </x:c>
       <x:c r="I14" s="8" t="str">
-        <x:v>Tokens (optional)</x:v>
-      </x:c>
-      <x:c r="J14" s="2"/>
-      <x:c r="K14" s="2"/>
+        <x:v>Total model tokens</x:v>
+      </x:c>
+      <x:c r="J14" s="30" t="str">
+        <x:v>Input tokens</x:v>
+      </x:c>
+      <x:c r="K14" s="30" t="str">
+        <x:v>Cached input tokens</x:v>
+      </x:c>
+      <x:c r="L14" s="31" t="str">
+        <x:v>Output tokens</x:v>
+      </x:c>
+      <x:c r="M14" s="31" t="str">
+        <x:v>Reasoning output tokens</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="2"/>
@@ -1860,14 +2744,36 @@
       <x:c r="C15" s="2" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D15" s="17"/>
-      <x:c r="E15" s="18"/>
-      <x:c r="F15" s="18"/>
-      <x:c r="G15" s="18"/>
-      <x:c r="H15" s="18"/>
-      <x:c r="I15" s="18"/>
-      <x:c r="J15" s="2"/>
-      <x:c r="K15" s="2"/>
+      <x:c r="D15" s="32" t="n">
+        <x:v>42.3280398</x:v>
+      </x:c>
+      <x:c r="E15" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F15" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G15" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H15" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" s="36" t="n">
+        <x:v>182967</x:v>
+      </x:c>
+      <x:c r="J15" s="36" t="n">
+        <x:v>181332</x:v>
+      </x:c>
+      <x:c r="K15" s="36" t="n">
+        <x:v>143232</x:v>
+      </x:c>
+      <x:c r="L15" s="37" t="n">
+        <x:v>1635</x:v>
+      </x:c>
+      <x:c r="M15" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="2"/>
@@ -1877,14 +2783,36 @@
       <x:c r="C16" s="2" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D16" s="17"/>
-      <x:c r="E16" s="18"/>
-      <x:c r="F16" s="18"/>
-      <x:c r="G16" s="18"/>
-      <x:c r="H16" s="18"/>
-      <x:c r="I16" s="18"/>
-      <x:c r="J16" s="2"/>
-      <x:c r="K16" s="2"/>
+      <x:c r="D16" s="32" t="n">
+        <x:v>6.123118199999997</x:v>
+      </x:c>
+      <x:c r="E16" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F16" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G16" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H16" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K16" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L16" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M16" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="2"/>
@@ -1894,14 +2822,36 @@
       <x:c r="C17" s="2" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D17" s="17"/>
-      <x:c r="E17" s="18"/>
-      <x:c r="F17" s="18"/>
-      <x:c r="G17" s="18"/>
-      <x:c r="H17" s="18"/>
-      <x:c r="I17" s="18"/>
-      <x:c r="J17" s="2"/>
-      <x:c r="K17" s="2"/>
+      <x:c r="D17" s="32" t="n">
+        <x:v>44.4053048</x:v>
+      </x:c>
+      <x:c r="E17" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F17" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G17" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H17" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="36" t="n">
+        <x:v>185533</x:v>
+      </x:c>
+      <x:c r="J17" s="36" t="n">
+        <x:v>183586</x:v>
+      </x:c>
+      <x:c r="K17" s="36" t="n">
+        <x:v>163968</x:v>
+      </x:c>
+      <x:c r="L17" s="37" t="n">
+        <x:v>1947</x:v>
+      </x:c>
+      <x:c r="M17" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="2"/>
@@ -1911,14 +2861,36 @@
       <x:c r="C18" s="2" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D18" s="17"/>
-      <x:c r="E18" s="18"/>
-      <x:c r="F18" s="18"/>
-      <x:c r="G18" s="18"/>
-      <x:c r="H18" s="18"/>
-      <x:c r="I18" s="18"/>
-      <x:c r="J18" s="2"/>
-      <x:c r="K18" s="2"/>
+      <x:c r="D18" s="32" t="n">
+        <x:v>6.096144200000002</x:v>
+      </x:c>
+      <x:c r="E18" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F18" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G18" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H18" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K18" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L18" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M18" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="2"/>
@@ -1928,14 +2900,36 @@
       <x:c r="C19" s="2" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D19" s="17"/>
-      <x:c r="E19" s="18"/>
-      <x:c r="F19" s="18"/>
-      <x:c r="G19" s="18"/>
-      <x:c r="H19" s="18"/>
-      <x:c r="I19" s="18"/>
-      <x:c r="J19" s="2"/>
-      <x:c r="K19" s="2"/>
+      <x:c r="D19" s="32" t="n">
+        <x:v>34.024773700000004</x:v>
+      </x:c>
+      <x:c r="E19" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F19" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G19" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H19" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="36" t="n">
+        <x:v>142184</x:v>
+      </x:c>
+      <x:c r="J19" s="36" t="n">
+        <x:v>141586</x:v>
+      </x:c>
+      <x:c r="K19" s="36" t="n">
+        <x:v>122880</x:v>
+      </x:c>
+      <x:c r="L19" s="37" t="n">
+        <x:v>598</x:v>
+      </x:c>
+      <x:c r="M19" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="2"/>
@@ -1945,14 +2939,36 @@
       <x:c r="C20" s="2" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D20" s="17"/>
-      <x:c r="E20" s="18"/>
-      <x:c r="F20" s="18"/>
-      <x:c r="G20" s="18"/>
-      <x:c r="H20" s="18"/>
-      <x:c r="I20" s="18"/>
-      <x:c r="J20" s="2"/>
-      <x:c r="K20" s="2"/>
+      <x:c r="D20" s="32" t="n">
+        <x:v>6.109858500000002</x:v>
+      </x:c>
+      <x:c r="E20" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F20" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G20" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H20" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J20" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K20" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L20" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M20" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
       <x:c r="A21" s="2"/>
@@ -1962,14 +2978,36 @@
       <x:c r="C21" s="2" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D21" s="17"/>
-      <x:c r="E21" s="18"/>
-      <x:c r="F21" s="18"/>
-      <x:c r="G21" s="18"/>
-      <x:c r="H21" s="18"/>
-      <x:c r="I21" s="18"/>
-      <x:c r="J21" s="2"/>
-      <x:c r="K21" s="2"/>
+      <x:c r="D21" s="32" t="n">
+        <x:v>29.247441099999996</x:v>
+      </x:c>
+      <x:c r="E21" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F21" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G21" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H21" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I21" s="36" t="n">
+        <x:v>115581</x:v>
+      </x:c>
+      <x:c r="J21" s="36" t="n">
+        <x:v>114274</x:v>
+      </x:c>
+      <x:c r="K21" s="36" t="n">
+        <x:v>104576</x:v>
+      </x:c>
+      <x:c r="L21" s="37" t="n">
+        <x:v>1307</x:v>
+      </x:c>
+      <x:c r="M21" s="37" t="n">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="2"/>
@@ -1979,14 +3017,36 @@
       <x:c r="C22" s="2" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D22" s="17"/>
-      <x:c r="E22" s="18"/>
-      <x:c r="F22" s="18"/>
-      <x:c r="G22" s="18"/>
-      <x:c r="H22" s="18"/>
-      <x:c r="I22" s="18"/>
-      <x:c r="J22" s="2"/>
-      <x:c r="K22" s="2"/>
+      <x:c r="D22" s="32" t="n">
+        <x:v>6.114583299999999</x:v>
+      </x:c>
+      <x:c r="E22" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F22" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G22" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H22" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I22" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J22" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K22" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L22" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M22" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" s="2"/>
@@ -1996,14 +3056,36 @@
       <x:c r="C23" s="2" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D23" s="17"/>
-      <x:c r="E23" s="18"/>
-      <x:c r="F23" s="18"/>
-      <x:c r="G23" s="18"/>
-      <x:c r="H23" s="18"/>
-      <x:c r="I23" s="18"/>
-      <x:c r="J23" s="2"/>
-      <x:c r="K23" s="2"/>
+      <x:c r="D23" s="32" t="n">
+        <x:v>37.72880859999999</x:v>
+      </x:c>
+      <x:c r="E23" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F23" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G23" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H23" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="36" t="n">
+        <x:v>118116</x:v>
+      </x:c>
+      <x:c r="J23" s="36" t="n">
+        <x:v>116178</x:v>
+      </x:c>
+      <x:c r="K23" s="36" t="n">
+        <x:v>83456</x:v>
+      </x:c>
+      <x:c r="L23" s="37" t="n">
+        <x:v>1938</x:v>
+      </x:c>
+      <x:c r="M23" s="37" t="n">
+        <x:v>17</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
       <x:c r="A24" s="2"/>
@@ -2013,14 +3095,36 @@
       <x:c r="C24" s="2" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D24" s="17"/>
-      <x:c r="E24" s="18"/>
-      <x:c r="F24" s="18"/>
-      <x:c r="G24" s="18"/>
-      <x:c r="H24" s="18"/>
-      <x:c r="I24" s="18"/>
-      <x:c r="J24" s="2"/>
-      <x:c r="K24" s="2"/>
+      <x:c r="D24" s="32" t="n">
+        <x:v>6.111938999999984</x:v>
+      </x:c>
+      <x:c r="E24" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F24" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G24" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H24" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J24" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K24" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M24" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
       <x:c r="A25" s="2"/>
@@ -2030,14 +3134,36 @@
       <x:c r="C25" s="2" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D25" s="17"/>
-      <x:c r="E25" s="18"/>
-      <x:c r="F25" s="18"/>
-      <x:c r="G25" s="18"/>
-      <x:c r="H25" s="18"/>
-      <x:c r="I25" s="18"/>
-      <x:c r="J25" s="2"/>
-      <x:c r="K25" s="2"/>
+      <x:c r="D25" s="32" t="n">
+        <x:v>35.83691159999999</x:v>
+      </x:c>
+      <x:c r="E25" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F25" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G25" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H25" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I25" s="36" t="n">
+        <x:v>116407</x:v>
+      </x:c>
+      <x:c r="J25" s="36" t="n">
+        <x:v>114822</x:v>
+      </x:c>
+      <x:c r="K25" s="36" t="n">
+        <x:v>82048</x:v>
+      </x:c>
+      <x:c r="L25" s="37" t="n">
+        <x:v>1585</x:v>
+      </x:c>
+      <x:c r="M25" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
       <x:c r="A26" s="2"/>
@@ -2047,14 +3173,36 @@
       <x:c r="C26" s="2" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D26" s="17"/>
-      <x:c r="E26" s="18"/>
-      <x:c r="F26" s="18"/>
-      <x:c r="G26" s="18"/>
-      <x:c r="H26" s="18"/>
-      <x:c r="I26" s="18"/>
-      <x:c r="J26" s="2"/>
-      <x:c r="K26" s="2"/>
+      <x:c r="D26" s="32" t="n">
+        <x:v>6.128204300000013</x:v>
+      </x:c>
+      <x:c r="E26" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F26" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G26" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H26" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I26" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J26" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K26" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L26" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M26" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
       <x:c r="A27" s="2"/>
@@ -2064,14 +3212,36 @@
       <x:c r="C27" s="2" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D27" s="17"/>
-      <x:c r="E27" s="18"/>
-      <x:c r="F27" s="18"/>
-      <x:c r="G27" s="18"/>
-      <x:c r="H27" s="18"/>
-      <x:c r="I27" s="18"/>
-      <x:c r="J27" s="2"/>
-      <x:c r="K27" s="2"/>
+      <x:c r="D27" s="32" t="n">
+        <x:v>35.66634939999998</x:v>
+      </x:c>
+      <x:c r="E27" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F27" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G27" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H27" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I27" s="36" t="n">
+        <x:v>118093</x:v>
+      </x:c>
+      <x:c r="J27" s="36" t="n">
+        <x:v>116177</x:v>
+      </x:c>
+      <x:c r="K27" s="36" t="n">
+        <x:v>97408</x:v>
+      </x:c>
+      <x:c r="L27" s="37" t="n">
+        <x:v>1916</x:v>
+      </x:c>
+      <x:c r="M27" s="37" t="n">
+        <x:v>15</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
       <x:c r="A28" s="2"/>
@@ -2081,14 +3251,36 @@
       <x:c r="C28" s="2" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D28" s="17"/>
-      <x:c r="E28" s="18"/>
-      <x:c r="F28" s="18"/>
-      <x:c r="G28" s="18"/>
-      <x:c r="H28" s="18"/>
-      <x:c r="I28" s="18"/>
-      <x:c r="J28" s="2"/>
-      <x:c r="K28" s="2"/>
+      <x:c r="D28" s="32" t="n">
+        <x:v>6.1226558000000075</x:v>
+      </x:c>
+      <x:c r="E28" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F28" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G28" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H28" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I28" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J28" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K28" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M28" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
       <x:c r="A29" s="2"/>
@@ -2098,14 +3290,36 @@
       <x:c r="C29" s="2" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D29" s="17"/>
-      <x:c r="E29" s="18"/>
-      <x:c r="F29" s="18"/>
-      <x:c r="G29" s="18"/>
-      <x:c r="H29" s="18"/>
-      <x:c r="I29" s="18"/>
-      <x:c r="J29" s="2"/>
-      <x:c r="K29" s="2"/>
+      <x:c r="D29" s="32" t="n">
+        <x:v>44.157766899999984</x:v>
+      </x:c>
+      <x:c r="E29" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F29" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G29" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H29" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I29" s="36" t="n">
+        <x:v>185326</x:v>
+      </x:c>
+      <x:c r="J29" s="36" t="n">
+        <x:v>183388</x:v>
+      </x:c>
+      <x:c r="K29" s="36" t="n">
+        <x:v>172800</x:v>
+      </x:c>
+      <x:c r="L29" s="37" t="n">
+        <x:v>1938</x:v>
+      </x:c>
+      <x:c r="M29" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
       <x:c r="A30" s="2"/>
@@ -2115,14 +3329,36 @@
       <x:c r="C30" s="2" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D30" s="17"/>
-      <x:c r="E30" s="18"/>
-      <x:c r="F30" s="18"/>
-      <x:c r="G30" s="18"/>
-      <x:c r="H30" s="18"/>
-      <x:c r="I30" s="18"/>
-      <x:c r="J30" s="2"/>
-      <x:c r="K30" s="2"/>
+      <x:c r="D30" s="32" t="n">
+        <x:v>6.1330272000000114</x:v>
+      </x:c>
+      <x:c r="E30" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F30" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G30" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H30" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J30" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K30" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M30" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="25" customHeight="1">
       <x:c r="A31" s="2"/>
@@ -2132,14 +3368,36 @@
       <x:c r="C31" s="2" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="D31" s="17"/>
-      <x:c r="E31" s="18"/>
-      <x:c r="F31" s="18"/>
-      <x:c r="G31" s="18"/>
-      <x:c r="H31" s="18"/>
-      <x:c r="I31" s="18"/>
-      <x:c r="J31" s="2"/>
-      <x:c r="K31" s="2"/>
+      <x:c r="D31" s="32" t="n">
+        <x:v>41.29774200000003</x:v>
+      </x:c>
+      <x:c r="E31" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F31" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G31" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H31" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I31" s="36" t="n">
+        <x:v>183042</x:v>
+      </x:c>
+      <x:c r="J31" s="36" t="n">
+        <x:v>181415</x:v>
+      </x:c>
+      <x:c r="K31" s="36" t="n">
+        <x:v>170880</x:v>
+      </x:c>
+      <x:c r="L31" s="37" t="n">
+        <x:v>1627</x:v>
+      </x:c>
+      <x:c r="M31" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="25" customHeight="1">
       <x:c r="A32" s="2"/>
@@ -2149,14 +3407,36 @@
       <x:c r="C32" s="2" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="D32" s="17"/>
-      <x:c r="E32" s="18"/>
-      <x:c r="F32" s="18"/>
-      <x:c r="G32" s="18"/>
-      <x:c r="H32" s="18"/>
-      <x:c r="I32" s="18"/>
-      <x:c r="J32" s="2"/>
-      <x:c r="K32" s="2"/>
+      <x:c r="D32" s="32" t="n">
+        <x:v>6.1259384000000425</x:v>
+      </x:c>
+      <x:c r="E32" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F32" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G32" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H32" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I32" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K32" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M32" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="25" customHeight="1">
       <x:c r="A33" s="2"/>
@@ -2166,14 +3446,36 @@
       <x:c r="C33" s="2" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D33" s="17"/>
-      <x:c r="E33" s="18"/>
-      <x:c r="F33" s="18"/>
-      <x:c r="G33" s="18"/>
-      <x:c r="H33" s="18"/>
-      <x:c r="I33" s="18"/>
-      <x:c r="J33" s="2"/>
-      <x:c r="K33" s="2"/>
+      <x:c r="D33" s="32" t="n">
+        <x:v>55.79296789999999</x:v>
+      </x:c>
+      <x:c r="E33" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F33" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G33" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H33" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I33" s="36" t="n">
+        <x:v>185795</x:v>
+      </x:c>
+      <x:c r="J33" s="36" t="n">
+        <x:v>183824</x:v>
+      </x:c>
+      <x:c r="K33" s="36" t="n">
+        <x:v>164224</x:v>
+      </x:c>
+      <x:c r="L33" s="37" t="n">
+        <x:v>1971</x:v>
+      </x:c>
+      <x:c r="M33" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="25" customHeight="1">
       <x:c r="A34" s="2"/>
@@ -2183,14 +3485,36 @@
       <x:c r="C34" s="2" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D34" s="17"/>
-      <x:c r="E34" s="18"/>
-      <x:c r="F34" s="18"/>
-      <x:c r="G34" s="18"/>
-      <x:c r="H34" s="18"/>
-      <x:c r="I34" s="18"/>
-      <x:c r="J34" s="2"/>
-      <x:c r="K34" s="2"/>
+      <x:c r="D34" s="32" t="n">
+        <x:v>6.167543500000029</x:v>
+      </x:c>
+      <x:c r="E34" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F34" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G34" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H34" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K34" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M34" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="2"/>
@@ -2221,7 +3545,7 @@
     <x:row r="37">
       <x:c r="A37" s="2"/>
       <x:c r="B37" s="2" t="str">
-        <x:v>Field accuracy = correct expected fields / total expected fields. Missing or wrong values are incorrect. Extra rows also fail task success.</x:v>
+        <x:v>Field accuracy counts 20 canonical expected values per trial, validated in BOTH CSV and JSON. Wrong/missing fields are incorrect.</x:v>
       </x:c>
       <x:c r="C37" s="2"/>
       <x:c r="D37" s="2"/>
@@ -2236,7 +3560,7 @@
     <x:row r="38">
       <x:c r="A38" s="2"/>
       <x:c r="B38" s="2" t="str">
-        <x:v>For the scraper, freeze ASIN, title, price and URL for all five unique rows: 20 expected fields per run.</x:v>
+        <x:v>Pairs 1–5: unchanged catalog. 6: price. 7: title. 8: missing optional price. 9: conflicting duplicate. 10: comma and HTML entity.</x:v>
       </x:c>
       <x:c r="C38" s="2"/>
       <x:c r="D38" s="2"/>
@@ -2251,7 +3575,7 @@
     <x:row r="39">
       <x:c r="A39" s="2"/>
       <x:c r="B39" s="2" t="str">
-        <x:v>Success requires the exact expected row set, valid values, the requested file and completion before the shared timeout.</x:v>
+        <x:v>All trials used the same prompt/graph and first-occurrence deduplication. No manual corrections or whole-trial retries.</x:v>
       </x:c>
       <x:c r="C39" s="2"/>
       <x:c r="D39" s="2"/>
@@ -2266,7 +3590,7 @@
     <x:row r="40">
       <x:c r="A40" s="2"/>
       <x:c r="B40" s="2" t="str">
-        <x:v>Speedup = prompt-agent mean time / workflow mean time. Values above 1 favor the workflow. Accuracy difference is workflow minus agent.</x:v>
+        <x:v>Timer includes method startup, both 3-second waits, execution, agent completion and file validation. Compilation/setup authoring excluded.</x:v>
       </x:c>
       <x:c r="C40" s="2"/>
       <x:c r="D40" s="2"/>
@@ -2281,7 +3605,7 @@
     <x:row r="41">
       <x:c r="A41" s="2"/>
       <x:c r="B41" s="2" t="str">
-        <x:v>Enter paired measurements for both methods before using results. Do not compare native scraping with unrelated AI-heavy tasks.</x:v>
+        <x:v>An independent Python CSV/JSON audit reproduced all 20 scores, fixture hashes and aggregate mean/median values.</x:v>
       </x:c>
       <x:c r="C41" s="2"/>
       <x:c r="D41" s="2"/>
@@ -2295,7 +3619,9 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="2"/>
-      <x:c r="B42" s="2"/>
+      <x:c r="B42" s="2" t="str">
+        <x:v>Agent: GPT-6.1 Sol, low reasoning, ChatGPT subscription. Reported tokens include cached input; they are not a dollar cost measure.</x:v>
+      </x:c>
       <x:c r="C42" s="2"/>
       <x:c r="D42" s="2"/>
       <x:c r="E42" s="2"/>
@@ -2308,7 +3634,9 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="2"/>
-      <x:c r="B43" s="2"/>
+      <x:c r="B43" s="2" t="str">
+        <x:v>Workflow: production runGraph/executeNativeStep with native Rust parsing and file writers. Tauri transport replaced by local stdio.</x:v>
+      </x:c>
       <x:c r="C43" s="2"/>
       <x:c r="D43" s="2"/>
       <x:c r="E43" s="2"/>
@@ -2321,7 +3649,9 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="2"/>
-      <x:c r="B44" s="2"/>
+      <x:c r="B44" s="2" t="str">
+        <x:v>These small frozen cases do not establish accuracy on other sites or speed for AI-heavy steps. Shared parser isolates orchestration.</x:v>
+      </x:c>
       <x:c r="C44" s="2"/>
       <x:c r="D44" s="2"/>
       <x:c r="E44" s="2"/>
@@ -2345,11 +3675,17 @@
       <x:c r="J45" s="2"/>
       <x:c r="K45" s="2"/>
     </x:row>
-    <x:row r="46">
+    <x:row r="46" ht="30" customHeight="1">
       <x:c r="A46" s="2"/>
-      <x:c r="B46" s="2"/>
-      <x:c r="C46" s="2"/>
-      <x:c r="D46" s="2"/>
+      <x:c r="B46" s="26" t="str">
+        <x:v>Mean token usage per run</x:v>
+      </x:c>
+      <x:c r="C46" s="26" t="str">
+        <x:v>Prompt agent</x:v>
+      </x:c>
+      <x:c r="D46" s="26" t="str">
+        <x:v>Workflow</x:v>
+      </x:c>
       <x:c r="E46" s="2"/>
       <x:c r="F46" s="2"/>
       <x:c r="G46" s="2"/>
@@ -2360,9 +3696,17 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2"/>
-      <x:c r="B47" s="2"/>
-      <x:c r="C47" s="2"/>
-      <x:c r="D47" s="2"/>
+      <x:c r="B47" s="2" t="str">
+        <x:v>Total model tokens</x:v>
+      </x:c>
+      <x:c r="C47" s="38" t="n">
+        <x:f>SUMIFS($I$15:$I$34,$B$15:$B$34,C$46)/COUNTIFS($B$15:$B$34,C$46)</x:f>
+        <x:v>153304.4</x:v>
+      </x:c>
+      <x:c r="D47" s="38" t="n">
+        <x:f>SUMIFS($I$15:$I$34,$B$15:$B$34,D$46)/COUNTIFS($B$15:$B$34,D$46)</x:f>
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E47" s="2"/>
       <x:c r="F47" s="2"/>
       <x:c r="G47" s="2"/>
@@ -2373,9 +3717,17 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2"/>
-      <x:c r="B48" s="2"/>
-      <x:c r="C48" s="2"/>
-      <x:c r="D48" s="2"/>
+      <x:c r="B48" s="2" t="str">
+        <x:v>Input tokens</x:v>
+      </x:c>
+      <x:c r="C48" s="38" t="n">
+        <x:f>SUMIFS($J$15:$J$34,$B$15:$B$34,C$46)/COUNTIFS($B$15:$B$34,C$46)</x:f>
+        <x:v>151658.2</x:v>
+      </x:c>
+      <x:c r="D48" s="38" t="n">
+        <x:f>SUMIFS($J$15:$J$34,$B$15:$B$34,D$46)/COUNTIFS($B$15:$B$34,D$46)</x:f>
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E48" s="2"/>
       <x:c r="F48" s="2"/>
       <x:c r="G48" s="2"/>
@@ -2386,9 +3738,17 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2"/>
-      <x:c r="B49" s="2"/>
-      <x:c r="C49" s="2"/>
-      <x:c r="D49" s="2"/>
+      <x:c r="B49" s="2" t="str">
+        <x:v>Cached input tokens</x:v>
+      </x:c>
+      <x:c r="C49" s="38" t="n">
+        <x:f>SUMIFS($K$15:$K$34,$B$15:$B$34,C$46)/COUNTIFS($B$15:$B$34,C$46)</x:f>
+        <x:v>130547.2</x:v>
+      </x:c>
+      <x:c r="D49" s="38" t="n">
+        <x:f>SUMIFS($K$15:$K$34,$B$15:$B$34,D$46)/COUNTIFS($B$15:$B$34,D$46)</x:f>
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E49" s="2"/>
       <x:c r="F49" s="2"/>
       <x:c r="G49" s="2"/>
@@ -2399,9 +3759,17 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="2"/>
-      <x:c r="B50" s="2"/>
-      <x:c r="C50" s="2"/>
-      <x:c r="D50" s="2"/>
+      <x:c r="B50" s="2" t="str">
+        <x:v>Output tokens</x:v>
+      </x:c>
+      <x:c r="C50" s="38" t="n">
+        <x:f>SUMIFS($L$15:$L$34,$B$15:$B$34,C$46)/COUNTIFS($B$15:$B$34,C$46)</x:f>
+        <x:v>1646.2</x:v>
+      </x:c>
+      <x:c r="D50" s="38" t="n">
+        <x:f>SUMIFS($L$15:$L$34,$B$15:$B$34,D$46)/COUNTIFS($B$15:$B$34,D$46)</x:f>
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E50" s="2"/>
       <x:c r="F50" s="2"/>
       <x:c r="G50" s="2"/>
@@ -2412,9 +3780,17 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="2"/>
-      <x:c r="B51" s="2"/>
-      <x:c r="C51" s="2"/>
-      <x:c r="D51" s="2"/>
+      <x:c r="B51" s="2" t="str">
+        <x:v>Reasoning output tokens</x:v>
+      </x:c>
+      <x:c r="C51" s="38" t="n">
+        <x:f>SUMIFS($M$15:$M$34,$B$15:$B$34,C$46)/COUNTIFS($B$15:$B$34,C$46)</x:f>
+        <x:v>4.4</x:v>
+      </x:c>
+      <x:c r="D51" s="38" t="n">
+        <x:f>SUMIFS($M$15:$M$34,$B$15:$B$34,D$46)/COUNTIFS($B$15:$B$34,D$46)</x:f>
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E51" s="2"/>
       <x:c r="F51" s="2"/>
       <x:c r="G51" s="2"/>
@@ -2438,7 +3814,9 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="2"/>
-      <x:c r="B53" s="2"/>
+      <x:c r="B53" s="2" t="str">
+        <x:v>Tokens are cumulative for the whole agent run. Total = input + output; cached input is included in input and is not added again.</x:v>
+      </x:c>
       <x:c r="C53" s="2"/>
       <x:c r="D53" s="2"/>
       <x:c r="E53" s="2"/>
@@ -2451,7 +3829,9 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="2"/>
-      <x:c r="B54" s="2"/>
+      <x:c r="B54" s="2" t="str">
+        <x:v>Native runs invoke no model. AI builder/setup and AI-heavy steps are excluded; zero here does not mean all workflows use zero tokens.</x:v>
+      </x:c>
       <x:c r="C54" s="2"/>
       <x:c r="D54" s="2"/>
       <x:c r="E54" s="2"/>

</xml_diff>